<commit_message>
Clean stale external links from Excel templates
</commit_message>
<xml_diff>
--- a/templates/관리번호스티커(서식).xlsx
+++ b/templates/관리번호스티커(서식).xlsx
@@ -15,10 +15,6 @@
   <sheets>
     <sheet name="관리번호스티커(서식)" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-    <externalReference r:id="rId3"/>
-  </externalReferences>
   <definedNames>
     <definedName name="DB등록여부">#REF!</definedName>
     <definedName name="DB등록여부2">[2]유효성검사!$G$3:$G$4</definedName>
@@ -144,138 +140,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="표지(서식)"/>
-      <sheetName val="기록물관리대장"/>
-      <sheetName val="신규"/>
-      <sheetName val="관리번호스티커(서식)"/>
-      <sheetName val="맞춤"/>
-      <sheetName val="양식"/>
-      <sheetName val="학교단위과제"/>
-      <sheetName val="충청남도교육청 기관별 명칭 및 기관코드"/>
-      <sheetName val="유효성검사"/>
-      <sheetName val="서식 1_일반기록물 생산현황(서식)"/>
-      <sheetName val="서식 3_시청각기록물 생산현황(서식)"/>
-      <sheetName val="서식 4_시청각기록물 생산목록(서식)"/>
-      <sheetName val="서식 7_회의록 생산현황(서식)"/>
-      <sheetName val="서식 8_회의록 생산목록(서식)"/>
-      <sheetName val="상자라벨(서식)"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="기록물등록 기록물철 일괄등록서식"/>
-      <sheetName val="충청남도교육청 기관별 명칭 및 기관코드"/>
-      <sheetName val="학교단위과제"/>
-      <sheetName val="유효성검사"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="5">
-          <cell r="L5" t="str">
-            <v/>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1">
-        <row r="4">
-          <cell r="B4" t="str">
-            <v>충청남도교육청</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2">
-        <row r="6">
-          <cell r="D6" t="str">
-            <v>1.기숙사운영</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="3">
-        <row r="3">
-          <cell r="A3" t="str">
-            <v>문서류</v>
-          </cell>
-          <cell r="E3" t="str">
-            <v>1등급</v>
-          </cell>
-          <cell r="G3" t="str">
-            <v>O</v>
-          </cell>
-          <cell r="J3" t="str">
-            <v>전체열람</v>
-          </cell>
-          <cell r="K3" t="str">
-            <v>공개</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>시청각류</v>
-          </cell>
-          <cell r="E4" t="str">
-            <v>2등급</v>
-          </cell>
-          <cell r="G4" t="str">
-            <v>X</v>
-          </cell>
-          <cell r="J4" t="str">
-            <v>목록열람</v>
-          </cell>
-          <cell r="K4" t="str">
-            <v>부분공개</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="E5" t="str">
-            <v>3등급</v>
-          </cell>
-          <cell r="J5" t="str">
-            <v>열람불가</v>
-          </cell>
-          <cell r="K5" t="str">
-            <v>비공개</v>
-          </cell>
-        </row>
-      </sheetData>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>